<commit_message>
Movilización: apply numbers and committee reviews (edge-case controls, empty-month fixed charge, scenarios generated in code, clearer labels, operational risks, TRM exposure)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsMRKE8hArHddZxwmwcNWn
</commit_message>
<xml_diff>
--- a/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
+++ b/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
@@ -1218,7 +1218,7 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>CORREGIR — En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Estimo ≈1.063 USD/h de equipos…</t>
+          <t>CORREGIR — En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Estimo ≈1.357 USD/h de flota m…</t>
         </is>
       </c>
     </row>
@@ -2856,7 +2856,7 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Estimo ≈1.063 USD/h de equipos (flota 0–5 km de p.1 a tarifa horaria de p.5) más ≈161 USD/h de nómina (430 M COP / 720 h), en total ≈2.681 USD/h. EC no tiene cláusula expresa, pero cobra aparte los turnos y el personal extra (carta p.2), así que el piso es 1.456 USD/h.</t>
+          <t>En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Estimo ≈1.357 USD/h de flota mínima (p.3) y 20 señalizadores a tarifa horaria de p.5, en total ≈2.813 USD/h con el taladro (cifra única del simulador, hoja Pendientes). EC no tiene cláusula expresa, pero cobra aparte los turnos y el personal extra (carta p.2), así que el piso es 1.456 USD/h.</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -2866,7 +2866,7 @@
       </c>
       <c r="I56" s="4" t="inlineStr">
         <is>
-          <t>NPT de movilización que anula el ahorro: PS ≈ 6,8 h por movilización (18.095/2.681); EC ≈ 12,7 h por movilización solo con taladro (18.451/1.456). Con las horas de la cotización (24 h), PS baja a ≈ 4,2 h.</t>
+          <t>NPT de movilización que anula el ahorro: PS ≈ 6,4 h por movilización (18.095/2.813); EC ≈ 12,7 h por movilización solo con taladro (18.451/1.456). Con las horas de la cotización (24 h), PS baja a ≈ 4,0 h.</t>
         </is>
       </c>
     </row>
@@ -3468,7 +3468,7 @@
       </c>
       <c r="F11" s="4" t="inlineStr">
         <is>
-          <t>≈2.681 USD/h (PS) y ≥1.456 USD/h (EC). Unas 6,8 h por movilización anulan el ahorro de PS.</t>
+          <t>≈2.813 USD/h (PS) y ≥1.456 USD/h (EC). Unas 6,4 h por movilización anulan el ahorro de PS.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Movilización: deck KPIs data-driven, audit workbooks aligned to current base
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsMRKE8hArHddZxwmwcNWn
</commit_message>
<xml_diff>
--- a/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
+++ b/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
@@ -547,6 +547,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="28" customHeight="1">
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>Nota: las cifras propias de esta auditoría se calcularon con las premisas de la Zona 2 (Truck Manager por movilización, sin bloqueos, perfil 2024) para poder compararlas con ella. Los resultados vigentes del ejercicio están en Simulador_Movilizacion_GRS110.xlsx, hoja Resumen.</t>
+        </is>
+      </c>
+    </row>
     <row r="4">
       <c r="B4" s="3" t="inlineStr">
         <is>
@@ -1331,8 +1338,9 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="B2:F2"/>
+    <mergeCell ref="B3:F3"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Movilización: final audit fixes (blocked month incl. Truck Manager, input validations, chart links, pros/cons table, recommendation slide, unified names, neutral wording, print setup)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsMRKE8hArHddZxwmwcNWn
</commit_message>
<xml_diff>
--- a/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
+++ b/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
@@ -658,7 +658,7 @@
       </c>
       <c r="F7" s="6" t="inlineStr">
         <is>
-          <t>CORREGIR — Los 15 de misma localización son dato de SierraCol, pero son el 43 %, frente al 33 % de los logs de 2024 (23/70) y el 24 % de 2025 (11/45). Que los 20 restantes estén todos en 0,1–5 km es un supuesto del Excel, no de SierraCol. En los logs, los tramos 5–10 y &gt;…</t>
+          <t>CORREGIR — Los 15 de misma localización son dato de SierraCol, pero son el 43 %, frente al 33 % de los logs de 2024 (23/70) y el 24 % de 2025 (11/45). Que los 20 restantes estén todos en 0,1–5 km es un supuesto del Excel, no de SierraCol (confirmado después por SierraCol…</t>
         </is>
       </c>
     </row>
@@ -1144,7 +1144,7 @@
       </c>
       <c r="F25" s="6" t="inlineStr">
         <is>
-          <t>CORREGIR — Bajo sus propias premisas lo reproduzco: AH121 = 1.192 ≥ 0 y AH122 = −15.080 (PS); AI127 = 26.345 y AI128 = −8.744 (EC).</t>
+          <t>CORREGIR — Bajo sus propias premisas se reproduce: AH121 = 1.192 ≥ 0 y AH122 = −15.080 (PS); AI127 = 26.345 y AI128 = −8.744 (EC).</t>
         </is>
       </c>
     </row>
@@ -1225,7 +1225,7 @@
       </c>
       <c r="F28" s="6" t="inlineStr">
         <is>
-          <t>CORREGIR — En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Estimo ≈1.357 USD/h de flota m…</t>
+          <t>CORREGIR — En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Se estima ≈1.357 USD/h de flot…</t>
         </is>
       </c>
     </row>
@@ -1376,7 +1376,7 @@
     <row r="2">
       <c r="B2" s="8" t="inlineStr">
         <is>
-          <t>'Su número' = valor de la celda de la Zona 2. 'Mi número' = recálculo independiente (✓ = reproducido al centavo). Cifras de campaña verificadas contra el simulador.</t>
+          <t>'Valor de la evaluación' = valor de la celda de la Zona 2. 'Valor recalculado' = recálculo independiente (✓ = reproducido al centavo).</t>
         </is>
       </c>
     </row>
@@ -1420,12 +1420,12 @@
       </c>
       <c r="H5" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I5" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -1511,12 +1511,12 @@
       </c>
       <c r="H9" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I9" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -1562,7 +1562,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="105" customHeight="1">
+    <row r="11" ht="135" customHeight="1">
       <c r="B11" s="4" t="inlineStr">
         <is>
           <t>Mezcla de la campaña (J16=15, J17=20, K17 "Dif. Loc" llevado a C58 = 0,1–5 km)</t>
@@ -1590,7 +1590,7 @@
       </c>
       <c r="G11" s="4" t="inlineStr">
         <is>
-          <t>Los 15 de misma localización son dato de SierraCol, pero son el 43 %, frente al 33 % de los logs de 2024 (23/70) y el 24 % de 2025 (11/45). Que los 20 restantes estén todos en 0,1–5 km es un supuesto del Excel, no de SierraCol. En los logs, los tramos 5–10 y &gt;10 km pesan el 38 % (18/47) de los movimientos a otra localización en 2024 y el 50 % (17/34) en 2025. Son justamente los tramos donde el tercerizado pierde a tarifa plena (E85 −5.911 · G85 −8.760 · G111 −880).</t>
+          <t>Los 15 de misma localización son dato de SierraCol, pero son el 43 %, frente al 33 % de los logs de 2024 (23/70) y el 24 % de 2025 (11/45). Que los 20 restantes estén todos en 0,1–5 km es un supuesto del Excel, no de SierraCol (confirmado después por SierraCol: los 20 pozos van a 0,1–5 km; queda solo como riesgo si la campaña cambia). En los logs, los tramos 5–10 y &gt;10 km pesan el 38 % (18/47) de los movimientos a otra localización en 2024 y el 50 % (17/34) en 2025. Son justamente los tramos donde el tercerizado pierde a tarifa plena (E85 −5.911 · G85 −8.760 · G111 −880).</t>
         </is>
       </c>
       <c r="H11" s="4" t="inlineStr">
@@ -1686,12 +1686,12 @@
       </c>
       <c r="H15" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I15" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -1903,12 +1903,12 @@
       </c>
       <c r="H22" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I22" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -2078,12 +2078,12 @@
       </c>
       <c r="H28" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I28" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -2211,12 +2211,12 @@
       </c>
       <c r="H33" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I33" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -2344,12 +2344,12 @@
       </c>
       <c r="H38" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I38" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -2435,12 +2435,12 @@
       </c>
       <c r="H42" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I42" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -2568,12 +2568,12 @@
       </c>
       <c r="H47" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I47" s="10" t="inlineStr">
         <is>
-          <t>Mi número (meses discretos, TM mensual)</t>
+          <t>Valor recalculado (meses discretos, TM mensual)</t>
         </is>
       </c>
     </row>
@@ -2701,12 +2701,12 @@
       </c>
       <c r="H52" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I52" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -2738,7 +2738,7 @@
       </c>
       <c r="G53" s="4" t="inlineStr">
         <is>
-          <t>Bajo sus propias premisas lo reproduzco: AH121 = 1.192 ≥ 0 y AH122 = −15.080 (PS); AI127 = 26.345 y AI128 = −8.744 (EC).</t>
+          <t>Bajo sus propias premisas se reproduce: AH121 = 1.192 ≥ 0 y AH122 = −15.080 (PS); AI127 = 26.345 y AI128 = −8.744 (EC).</t>
         </is>
       </c>
       <c r="H53" s="4" t="inlineStr">
@@ -2864,7 +2864,7 @@
       </c>
       <c r="G56" s="4" t="inlineStr">
         <is>
-          <t>En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Estimo ≈1.357 USD/h de flota mínima (p.3) y 20 señalizadores a tarifa horaria de p.5, en total ≈2.813 USD/h con el taladro (cifra única del simulador, hoja Pendientes). EC no tiene cláusula expresa, pero cobra aparte los turnos y el personal extra (carta p.2), así que el piso es 1.456 USD/h.</t>
+          <t>En el WO no se pagan horas de taladro. En el tercerizado, cada hora de demora cuesta 1.456 USD de taladro. En PS se suma la cláusula 7 (Cot. p.5): si la demora no es atribuible al transportador, el cliente asume equipos y nómina. Se estima ≈1.357 USD/h de flota mínima (p.3) y 20 señalizadores a tarifa horaria de p.5, en total ≈2.813 USD/h con el taladro (cifra única del simulador, hoja Pendientes). EC no tiene cláusula expresa, pero cobra aparte los turnos y el personal extra (carta p.2), así que el piso es 1.456 USD/h.</t>
         </is>
       </c>
       <c r="H56" s="4" t="inlineStr">
@@ -2960,12 +2960,12 @@
       </c>
       <c r="H60" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I60" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -3051,12 +3051,12 @@
       </c>
       <c r="H64" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I64" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>
@@ -3142,12 +3142,12 @@
       </c>
       <c r="H68" s="10" t="inlineStr">
         <is>
-          <t>Su número</t>
+          <t>Valor de la evaluación</t>
         </is>
       </c>
       <c r="I68" s="10" t="inlineStr">
         <is>
-          <t>Mi número</t>
+          <t>Valor recalculado</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Movilización: last wording consistency fixes
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01BsMRKE8hArHddZxwmwcNWn
</commit_message>
<xml_diff>
--- a/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
+++ b/movilizacion/entregables/Auditoria_Evaluacion_Previa.xlsx
@@ -901,7 +901,7 @@
       </c>
       <c r="F16" s="5" t="inlineStr">
         <is>
-          <t>CONSERVAR — K83:K86 = E25, E51, E77, E103, que coinciden con las tarifas base de la Cot. p.1–2. L = 50 % (p.2). Que el 50 % se aplique a la tarifa base (PS normal) coincide con la evaluación principal de SierraCol.</t>
+          <t>CONSERVAR — K83:K86 = E25, E51, E77, E103, que coinciden con las tarifas base de la Cot. p.1–2. L = 50 % (p.2). Que el 50 % se aplique a la tarifa base (Petro Star tarifa normal) coincide con la evaluación principal de SierraCol.</t>
         </is>
       </c>
     </row>
@@ -1369,7 +1369,7 @@
     <row r="1">
       <c r="B1" s="1" t="inlineStr">
         <is>
-          <t>Detalle sección por sección: evidencia, su número y mi número</t>
+          <t>Detalle sección por sección: evidencia, valor de la evaluación y valor recalculado</t>
         </is>
       </c>
     </row>
@@ -2087,7 +2087,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="45" customHeight="1">
+    <row r="29" ht="60" customHeight="1">
       <c r="B29" s="4" t="inlineStr">
         <is>
           <t>PS plena y al 50 %</t>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="G29" s="4" t="inlineStr">
         <is>
-          <t>K83:K86 = E25, E51, E77, E103, que coinciden con las tarifas base de la Cot. p.1–2. L = 50 % (p.2). Que el 50 % se aplique a la tarifa base (PS normal) coincide con la evaluación principal de SierraCol.</t>
+          <t>K83:K86 = E25, E51, E77, E103, que coinciden con las tarifas base de la Cot. p.1–2. L = 50 % (p.2). Que el 50 % se aplique a la tarifa base (Petro Star tarifa normal) coincide con la evaluación principal de SierraCol.</t>
         </is>
       </c>
       <c r="H29" s="4" t="inlineStr">
@@ -3088,7 +3088,7 @@
       </c>
       <c r="G65" s="4" t="inlineStr">
         <is>
-          <t>(a) El rótulo engaña: no es una "prueba de estrés", sino la lectura más favorable del LS. (b) Los insumos F25 y F51 no coinciden con la Cot. 1255 (sección 2). (c) Hereda los meses fraccionarios. (d) No muestra el LS sin descuento por frecuencia, que es la evaluación principal. La conclusión de J185 (LS por debajo de la ruta base) se sostiene aun con las tarifas de la cotización: LS con descuento en el perfil de 2024 da 587.181, frente a 730.502 de PS normal.</t>
+          <t>(a) El rótulo engaña: no es una "prueba de estrés", sino la lectura más favorable del LS. (b) Los insumos F25 y F51 no coinciden con la Cot. 1255 (sección 2). (c) Hereda los meses fraccionarios. (d) No muestra el LS sin descuento por frecuencia, que es la evaluación principal. La conclusión de J185 (LS por debajo de la ruta base) se sostiene aun con las tarifas de la cotización: LS con descuento en el perfil de 2024 da 587.181, frente a 730.502 de Petro Star tarifa normal.</t>
         </is>
       </c>
       <c r="H65" s="4" t="inlineStr">
@@ -3363,7 +3363,7 @@
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Favorece WO (y a PS normal frente a LS)</t>
+          <t>Favorece WO (y a Petro Star tarifa normal frente a LS)</t>
         </is>
       </c>
       <c r="F7" s="4" t="inlineStr">

</xml_diff>